<commit_message>
Custom Roles: resolve section 3658 stubs - move 2 valid cases into 3527 sub-sections, leave 5 for QA decision
Per QA-lead ruling on the 7 remaining section-3658 stub cases:
- MOVED + reworded build-accurate + pushed to TestRail (200/200):
  C27731 -> 3549 Migration (legacy Owner -> Administrator; Blocked-UI)
  C27736 -> 3545 View and Manage AP/AR Data (corrected build-wrong label to
    'View and Manage AP/AR Data'; VIU-Verified from build chunk)
- LEFT in 3658 for QA-lead decision (not valid - redundant or build-wrong):
  C27729, C27730, C27732, C27734, C27738
Nothing deleted; all 7 remain snapshotted (reversible). No staging role/settings
changes. Regenerated CustomRoles_WordingVIU workbook (254 rows) + Blockers Tracker;
audit log + section-3658-resolution-2026-07-13.md added.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/custom-roles-run/CustomRoles_WordingVIU_2026-07-13.xlsx
+++ b/build/custom-roles-run/CustomRoles_WordingVIU_2026-07-13.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -476,178 +476,163 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Section 3658 dedupe: 3 duplicates deleted (C27735, C27733, C27737); 7 flagged for ruling.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+          <t>Section 3658 dedupe: 3 duplicates deleted (C27735, C27733, C27737).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Section 3658 resolution 2026-07-13: 2 valid stubs MOVED into 3527 sub-sections + reworded/pushed (C27731-&gt;3549 Migration, C27736-&gt;3545 View and Manage AP/AR Data); 5 left in 3658 for QA-lead decision (C27729, C27730, C27732, C27734, C27738 - redundant or build-wrong). See section-3658-resolution-2026-07-13.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>203</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Blocked-UI</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>38</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Deviation/Finding</t>
+          <t>Blocked-UI</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>11</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Deviation/Finding</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B12" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="B13" s="3" t="n">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Blocked-UI</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Deviation/Finding</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Roles List Page (3528)</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>18</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Create Custom Role (3529)</t>
+          <t>Roles List Page (3528)</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Edit Role (3530)</t>
+          <t>Create Custom Role (3529)</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Delete Role (3531)</t>
+          <t>Edit Role (3530)</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
@@ -659,20 +644,20 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Permission Summary (3532)</t>
+          <t>Delete Role (3531)</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -687,14 +672,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CRUD Cascade Rules (3533)</t>
+          <t>Permission Summary (3532)</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -703,61 +688,61 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Work Orders Permissions (3534)</t>
+          <t>CRUD Cascade Rules (3533)</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Work Order Lines Permissions (3535)</t>
+          <t>Work Orders Permissions (3534)</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Schedule Permissions (3536)</t>
+          <t>Work Order Lines Permissions (3535)</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C23" t="n">
         <v>3</v>
@@ -769,20 +754,20 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Customer Management Permissions (3537)</t>
+          <t>Schedule Permissions (3536)</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -791,20 +776,20 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Parts Department Permissions (3538)</t>
+          <t>Customer Management Permissions (3537)</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -813,64 +798,64 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Invoicing and Payments Permissions (3539)</t>
+          <t>Parts Department Permissions (3538)</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C26" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Timesheets Permissions (3540)</t>
+          <t>Invoicing and Payments Permissions (3539)</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>6</v>
       </c>
       <c r="C27" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" t="n">
         <v>1</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Page Access Toggles (3541)</t>
+          <t>Timesheets Permissions (3540)</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -879,20 +864,20 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Settings Access (3542)</t>
+          <t>Page Access Toggles (3541)</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -901,64 +886,64 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>View Mode (3543)</t>
+          <t>Settings Access (3542)</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>See Financial Data (3544)</t>
+          <t>View Mode (3543)</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>View and Manage AP/AR Data (3545)</t>
+          <t>See Financial Data (3544)</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>10</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
@@ -967,20 +952,20 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>View History Logs (3546)</t>
+          <t>View and Manage AP/AR Data (3545)</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -989,20 +974,20 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Staff Page Role Assignment (3547)</t>
+          <t>View History Logs (3546)</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -1011,20 +996,20 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Per-Role Verification (3548)</t>
+          <t>Staff Page Role Assignment (3547)</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -1033,13 +1018,13 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Migration (3549)</t>
+          <t>Per-Role Verification (3548)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1061,14 +1046,14 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Staff Record Settings (3550)</t>
+          <t>Migration (3549)</t>
         </is>
       </c>
       <c r="B37" t="n">
+        <v>12</v>
+      </c>
+      <c r="C37" t="n">
         <v>1</v>
-      </c>
-      <c r="C37" t="n">
-        <v>2</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -1077,23 +1062,23 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>QuickBooks Relocation (3551)</t>
+          <t>Staff Record Settings (3550)</t>
         </is>
       </c>
       <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" t="n">
         <v>0</v>
-      </c>
-      <c r="C38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" t="n">
-        <v>3</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
@@ -1105,33 +1090,33 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>User Feedback Strings (3552)</t>
+          <t>QuickBooks Relocation (3551)</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Cross-Permission Combinations (3553)</t>
+          <t>User Feedback Strings (3552)</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C40" t="n">
         <v>1</v>
@@ -1143,6 +1128,28 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Cross-Permission Combinations (3553)</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>9</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1157,7 +1164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H204"/>
+  <dimension ref="A1:H205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7535,25 +7542,25 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>C26488</t>
+          <t>C27736</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26488</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/27736</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>3546</v>
+        <v>3545</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>View History Logs</t>
+          <t>View and Manage AP/AR Data</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>View History Logs ON: work order history and line history are visible (work orders only)</t>
+          <t>The AP/AR cross-cutting toggle is labeled 'View and Manage AP/AR Data'</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -7568,19 +7575,19 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>UI (role with View History Logs ON): the WO detail shows the History (15) tab exposing work order + line history/change events. screenshot hist-HistOn.</t>
+          <t>Moved from stub section 3663 into 3545 (distinct structural check: 3545 had no toggle-label case; parallels the SFD toggle-exists case). Original stub claimed the label 'Manage Accounts Payable and Receivable' - BUILD-WRONG; corrected to the live build label. LABEL VIU-VERIFIED from the shipped build chunk CrossTogglesSection.ChT56hCk.js: 'Cross-Cutting Toggles' card contains 'See Financial Data', 'View and Manage AP/AR Data' (seeApArData), 'View History Logs'.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>C26489</t>
+          <t>C26488</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26489</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26488</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -7593,7 +7600,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>View History Logs OFF: work order history and line history are hidden (work orders only)</t>
+          <t>View History Logs ON: work order history and line history are visible (work orders only)</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -7608,32 +7615,32 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>UI (role with View History Logs OFF = Time Clock User): the WO detail has NO History tab (Lines/Notes/Timesheets/Stats only) — work order and line history are hidden. screenshot hist-HistOff.</t>
+          <t>UI (role with View History Logs ON): the WO detail shows the History (15) tab exposing work order + line history/change events. screenshot hist-HistOn.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>C26492</t>
+          <t>C26489</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26492</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26489</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>3547</v>
+        <v>3546</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Staff Page Role Assignment</t>
+          <t>View History Logs</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Changing a user's role logs them out immediately</t>
+          <t>View History Logs OFF: work order history and line history are hidden (work orders only)</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -7648,19 +7655,19 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>API/session: changing a user role logs them out immediately — the prior session is invalidated (409 Session has expired) right after the change.</t>
+          <t>UI (role with View History Logs OFF = Time Clock User): the WO detail has NO History tab (Lines/Notes/Timesheets/Stats only) — work order and line history are hidden. screenshot hist-HistOff.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>C26494</t>
+          <t>C26492</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26494</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26492</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -7673,7 +7680,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>A logged-in user is logged out immediately when their role changes</t>
+          <t>Changing a user's role logs them out immediately</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -7688,32 +7695,32 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>API/session: a logged-in user is logged out immediately when their role changes (session invalidated -&gt; 409 on next request).</t>
+          <t>API/session: changing a user role logs them out immediately — the prior session is invalidated (409 Session has expired) right after the change.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>C26495</t>
+          <t>C26494</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26495</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26494</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>3548</v>
+        <v>3547</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Per-Role Verification</t>
+          <t>Staff Page Role Assignment</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Administrator: role permissions match the expected set</t>
+          <t>A logged-in user is logged out immediately when their role changes</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -7723,24 +7730,24 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>Roles-API-Verified (permission set matches the live role); workflow spot-checks Blocked-UI</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Administrator permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>API/session: a logged-in user is logged out immediately when their role changes (session invalidated -&gt; 409 on next request).</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>C26496</t>
+          <t>C26495</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26496</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26495</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -7753,7 +7760,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Service Manager: role permissions match the expected set</t>
+          <t>Administrator: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -7768,19 +7775,19 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Service Manager permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Administrator permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>C26497</t>
+          <t>C26496</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26497</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26496</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -7793,7 +7800,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Senior Service Advisor: role permissions match the expected set</t>
+          <t>Service Manager: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -7808,19 +7815,19 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Senior Service Advisor permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Service Manager permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>C26498</t>
+          <t>C26497</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26498</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26497</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -7833,7 +7840,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Service Advisor: role permissions match the expected set</t>
+          <t>Senior Service Advisor: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -7848,19 +7855,19 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Service Advisor permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Senior Service Advisor permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>C26499</t>
+          <t>C26498</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26499</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26498</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -7873,7 +7880,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Foreman: role permissions match the expected set</t>
+          <t>Service Advisor: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -7888,19 +7895,19 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Foreman permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Service Advisor permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>C26500</t>
+          <t>C26499</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26500</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26499</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -7913,7 +7920,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Technician: role permissions match the expected set</t>
+          <t>Foreman: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -7928,19 +7935,19 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Technician permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Foreman permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>C26501</t>
+          <t>C26500</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26501</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26500</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -7953,7 +7960,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Parts Manager: role permissions match the expected set</t>
+          <t>Technician: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -7968,19 +7975,19 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Parts Manager permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Technician permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>C26502</t>
+          <t>C26501</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26502</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26501</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -7993,7 +8000,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Parts Technician: role permissions match the expected set</t>
+          <t>Parts Manager: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -8008,19 +8015,19 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Parts Technician permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Parts Manager permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>C26503</t>
+          <t>C26502</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26503</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26502</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -8033,7 +8040,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Office User: role permissions match the expected set</t>
+          <t>Parts Technician: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -8048,19 +8055,19 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Office User permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Parts Technician permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>C26504</t>
+          <t>C26503</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26504</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26503</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -8073,7 +8080,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Sales Representative: role permissions match the expected set</t>
+          <t>Office User: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -8088,19 +8095,19 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Sales Representative permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Office User permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>C26505</t>
+          <t>C26504</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26505</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26504</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -8113,7 +8120,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Time Clock User: role permissions match the expected set</t>
+          <t>Sales Representative: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -8128,19 +8135,19 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Time Clock User permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Sales Representative permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>C26506</t>
+          <t>C26505</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26506</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26505</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -8153,7 +8160,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Customer portal is on by default only for Service Advisor, Senior Service Advisor, Service Manager and Parts Manager (and Administrator)</t>
+          <t>Time Clock User: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -8163,37 +8170,37 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Roles-API-Verified (matches live per-role customerPortalPageAccess)</t>
+          <t>Roles-API-Verified (permission set matches the live role); workflow spot-checks Blocked-UI</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>customerPortalPageAccess per role confirmed live: on for Admin/SM/SSA/SA/PM; off for the rest (roles-matrix-2026-07-13).</t>
+          <t>Time Clock User permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>C26510</t>
+          <t>C26506</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26510</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26506</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>3549</v>
+        <v>3548</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Per-Role Verification</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Legacy 'Admin / Administrator' users become 'Administrator' after migration</t>
+          <t>Customer portal is on by default only for Service Advisor, Senior Service Advisor, Service Manager and Parts Manager (and Administrator)</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -8203,24 +8210,24 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Roles-API-Verified (matches live per-role customerPortalPageAccess)</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>Live roles API: destination system role exists = "Admin" (build name; case prose says Administrator), isEditable=true, 89 users, 42 perms. Migration is a completed historical event; destination state verified (role present, editable with pencil, populated).</t>
+          <t>customerPortalPageAccess per role confirmed live: on for Admin/SM/SSA/SA/PM; off for the rest (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>C26511</t>
+          <t>C26510</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26511</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26510</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -8233,7 +8240,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Legacy 'Office' users become 'Office User' after migration</t>
+          <t>Legacy 'Admin / Administrator' users become 'Administrator' after migration</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -8248,19 +8255,19 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Live roles API: "Office User" exists, isEditable=false (lock + eye only), 5 users, 23 perms — matches legacy Office -&gt; Office User destination.</t>
+          <t>Live roles API: destination system role exists = "Admin" (build name; case prose says Administrator), isEditable=true, 89 users, 42 perms. Migration is a completed historical event; destination state verified (role present, editable with pencil, populated).</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>C26512</t>
+          <t>C26511</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26512</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26511</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -8273,7 +8280,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Legacy 'Time Clock' users become 'Time Clock User' after migration</t>
+          <t>Legacy 'Office' users become 'Office User' after migration</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -8288,19 +8295,19 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Live roles API: "Time Clock User" exists, isEditable=false (lock + eye only), 11 users, 3 perms — matches legacy Time Clock -&gt; Time Clock User.</t>
+          <t>Live roles API: "Office User" exists, isEditable=false (lock + eye only), 5 users, 23 perms — matches legacy Office -&gt; Office User destination.</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>C26513</t>
+          <t>C26512</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26513</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26512</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -8313,7 +8320,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Legacy 'Service Manager' users become 'Service Manager' after migration</t>
+          <t>Legacy 'Time Clock' users become 'Time Clock User' after migration</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -8328,19 +8335,19 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Live roles API: "Service Manager" exists, isEditable=true, 3 users, 35 perms.</t>
+          <t>Live roles API: "Time Clock User" exists, isEditable=false (lock + eye only), 11 users, 3 perms — matches legacy Time Clock -&gt; Time Clock User.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>C26514</t>
+          <t>C26513</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26514</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26513</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -8353,7 +8360,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Legacy 'Senior Service Advisor' users become 'Senior Service Advisor' after migration</t>
+          <t>Legacy 'Service Manager' users become 'Service Manager' after migration</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -8368,19 +8375,19 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Live roles API: "Senior Service Advisor" exists, isEditable=true, 8 users, 32 perms.</t>
+          <t>Live roles API: "Service Manager" exists, isEditable=true, 3 users, 35 perms.</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>C26515</t>
+          <t>C26514</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26515</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26514</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -8393,7 +8400,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Legacy 'Service Advisor' users become 'Service Advisor' after migration</t>
+          <t>Legacy 'Senior Service Advisor' users become 'Senior Service Advisor' after migration</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -8408,19 +8415,19 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>Live roles API: "Service Advisor" exists, isEditable=true, 2 users, 26 perms.</t>
+          <t>Live roles API: "Senior Service Advisor" exists, isEditable=true, 8 users, 32 perms.</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>C26516</t>
+          <t>C26515</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26516</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26515</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -8433,7 +8440,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Legacy 'Foreman' users become 'Foreman' after migration</t>
+          <t>Legacy 'Service Advisor' users become 'Service Advisor' after migration</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -8448,19 +8455,19 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>Live roles API: "Foreman" exists, isEditable=true, 16 users, 23 perms.</t>
+          <t>Live roles API: "Service Advisor" exists, isEditable=true, 2 users, 26 perms.</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>C26517</t>
+          <t>C26516</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26517</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26516</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -8473,7 +8480,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Legacy 'Technician' users become 'Technician' after migration</t>
+          <t>Legacy 'Foreman' users become 'Foreman' after migration</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -8488,19 +8495,19 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>Live roles API: "Technician" exists, isEditable=true, 66 users, 6 perms, view_mode tech (confirmed via role detail) — matches legacy Technician destination.</t>
+          <t>Live roles API: "Foreman" exists, isEditable=true, 16 users, 23 perms.</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>C26518</t>
+          <t>C26517</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26518</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26517</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -8513,7 +8520,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Legacy 'Parts Manager' users become 'Parts Manager' after migration</t>
+          <t>Legacy 'Technician' users become 'Technician' after migration</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -8528,19 +8535,19 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>Live roles API: "Parts Manager" exists, isEditable=true, 4 users, 31 perms.</t>
+          <t>Live roles API: "Technician" exists, isEditable=true, 66 users, 6 perms, view_mode tech (confirmed via role detail) — matches legacy Technician destination.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>C26519</t>
+          <t>C26518</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26519</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26518</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -8553,7 +8560,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Legacy 'Parts Tech / Parts Technician' users become 'Parts Technician' after migration</t>
+          <t>Legacy 'Parts Manager' users become 'Parts Manager' after migration</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -8568,19 +8575,19 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>Live roles API: "Parts Technician" exists, isEditable=true, 10 users, 19 perms — matches legacy Parts Tech -&gt; Parts Technician.</t>
+          <t>Live roles API: "Parts Manager" exists, isEditable=true, 4 users, 31 perms.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>C26520</t>
+          <t>C26519</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26520</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26519</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -8593,7 +8600,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Legacy 'Sales Representative' users become 'Sales Representative' after migration</t>
+          <t>Legacy 'Parts Tech / Parts Technician' users become 'Parts Technician' after migration</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -8608,19 +8615,19 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>Live roles API: "Sales Representative" exists, isEditable=true, 15 users, 4 perms.</t>
+          <t>Live roles API: "Parts Technician" exists, isEditable=true, 10 users, 19 perms — matches legacy Parts Tech -&gt; Parts Technician.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>C26525</t>
+          <t>C26520</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26525</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26520</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -8633,7 +8640,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Changing a user's role logs that user out and forces them to log in again</t>
+          <t>Legacy 'Sales Representative' users become 'Sales Representative' after migration</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -8648,32 +8655,32 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>UI/API: after an admin changed the Tech user role, the user existing session returned 409 "Session has expired." on the next call — the role change logs the user out and forces re-login.</t>
+          <t>Live roles API: "Sales Representative" exists, isEditable=true, 15 users, 4 perms.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>C26528</t>
+          <t>C26525</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26528</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26525</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>3550</v>
+        <v>3549</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Staff Record Settings</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>The universal clock in / out is available to any active staff member, whatever their role</t>
+          <t>Changing a user's role logs that user out and forces them to log in again</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -8688,32 +8695,32 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>UI: the universal Clock In control appears in the top bar for every role observed (Admin, Technician, Time Clock User) — available to any active staff member whatever their role.</t>
+          <t>UI/API: after an admin changed the Tech user role, the user existing session returned 409 "Session has expired." on the next call — the role change logs the user out and forces re-login.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>C26532</t>
+          <t>C26528</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26532</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26528</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>3552</v>
+        <v>3550</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>User Feedback Strings</t>
+          <t>Staff Record Settings</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Create success message wording</t>
+          <t>The universal clock in / out is available to any active staff member, whatever their role</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -8723,24 +8730,24 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Verified-Label (build)</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>'Role created successfully.' confirmed in build.</t>
+          <t>UI: the universal Clock In control appears in the top bar for every role observed (Admin, Technician, Time Clock User) — available to any active staff member whatever their role.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>C26533</t>
+          <t>C26532</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26533</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26532</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -8753,7 +8760,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Update success message wording</t>
+          <t>Create success message wording</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -8768,19 +8775,19 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>'Role updated successfully.' confirmed in build.</t>
+          <t>'Role created successfully.' confirmed in build.</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>C26534</t>
+          <t>C26533</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26534</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26533</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -8793,7 +8800,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Deleting a custom role with 0 users shows a confirmation dialog</t>
+          <t>Update success message wording</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -8803,24 +8810,24 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Verified-Label (build)</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>UI: deleting a 0-user custom role opens dialog "Confirmation — Are you sure you want to delete this role? This action cannot be undone." [Cancel|Delete]. screenshot delete-confirm-dialog.</t>
+          <t>'Role updated successfully.' confirmed in build.</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>C26535</t>
+          <t>C26534</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26535</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26534</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -8833,7 +8840,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Deleting a custom role that has users is blocked</t>
+          <t>Deleting a custom role with 0 users shows a confirmation dialog</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -8848,19 +8855,19 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>UI: a custom role with users (Parth Cust1, 1 user) has no Delete option in its 3-dot menu — deletion is blocked.</t>
+          <t>UI: deleting a 0-user custom role opens dialog "Confirmation — Are you sure you want to delete this role? This action cannot be undone." [Cancel|Delete]. screenshot delete-confirm-dialog.</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>C26536</t>
+          <t>C26535</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26536</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26535</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -8873,7 +8880,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Turning See Financial Data on shows a confirmation dialog</t>
+          <t>Deleting a custom role that has users is blocked</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -8883,24 +8890,24 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Verified-Label (build)</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>'Enable See Financial Data?' + Cancel/Enable confirmed in build (FinancialDataConfirmModal).</t>
+          <t>UI: a custom role with users (Parth Cust1, 1 user) has no Delete option in its 3-dot menu — deletion is blocked.</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>C26537</t>
+          <t>C26536</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26537</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26536</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -8913,7 +8920,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Creating a role with no name is blocked with a required-field error</t>
+          <t>Turning See Financial Data on shows a confirmation dialog</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -8923,24 +8930,24 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Verified-Label (build)</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>UI: creating a role with no name is blocked — Create disabled and inline "Role name is a required field" error when the field is touched/cleared.</t>
+          <t>'Enable See Financial Data?' + Cancel/Enable confirmed in build (FinancialDataConfirmModal).</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>C26538</t>
+          <t>C26537</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26538</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26537</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -8953,7 +8960,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Creating a role with the same permissions as an existing role shows a 'similar role' warning</t>
+          <t>Creating a role with no name is blocked with a required-field error</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -8968,32 +8975,32 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>UI: creating a role with the same permissions as an existing role shows "Similar role already exists" warning with "Create Anyway" (SimilarRoleWarningModal, keyed on identical permissions).</t>
+          <t>UI: creating a role with no name is blocked — Create disabled and inline "Role name is a required field" error when the field is touched/cleared.</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>C26540</t>
+          <t>C26538</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26540</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26538</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>3553</v>
+        <v>3552</v>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Cross-Permission Combinations</t>
+          <t>User Feedback Strings</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>A role with all permissions off blocks the user from every feature</t>
+          <t>Creating a role with the same permissions as an existing role shows a 'similar role' warning</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -9008,19 +9015,19 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>UI: a near-minimal custom role (only scheduleView) shows a minimal nav (just Schedule + Clock In); navigating to /reports or /administration/staff is refused and redirects to /schedule. (A truly all-off role cannot be saved — Create is disabled at zero perms, C26335 — so the practical minimum is one feature perm; that user is blocked from every other feature.) screenshot xperm-MinRole.</t>
+          <t>UI: creating a role with the same permissions as an existing role shows "Similar role already exists" warning with "Create Anyway" (SimilarRoleWarningModal, keyed on identical permissions).</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>C26541</t>
+          <t>C26540</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26541</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26540</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -9033,7 +9040,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>A role with all permissions on behaves like Administrator but is still a custom role</t>
+          <t>A role with all permissions off blocks the user from every feature</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
@@ -9048,19 +9055,19 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>UI: an all-permissions custom role (42 perms, all cross-toggles on, type Custom) behaves like Administrator — full nav (Work Orders/Schedule/Customers/Parts/Reports), /reports and /administration/staff accessible — yet it is a Custom role (created via Create Custom Role). screenshot xperm-AllOn.</t>
+          <t>UI: a near-minimal custom role (only scheduleView) shows a minimal nav (just Schedule + Clock In); navigating to /reports or /administration/staff is refused and redirects to /schedule. (A truly all-off role cannot be saved — Create is disabled at zero perms, C26335 — so the practical minimum is one feature perm; that user is blocked from every other feature.) screenshot xperm-MinRole.</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>C26542</t>
+          <t>C26541</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26542</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26541</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -9073,7 +9080,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>A system role cannot be deleted</t>
+          <t>A role with all permissions on behaves like Administrator but is still a custom role</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -9083,24 +9090,24 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Roles-API-Verified (all system roles deletable=false)</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>deletable=false for all system roles (live roles API).</t>
+          <t>UI: an all-permissions custom role (42 perms, all cross-toggles on, type Custom) behaves like Administrator — full nav (Work Orders/Schedule/Customers/Parts/Reports), /reports and /administration/staff accessible — yet it is a Custom role (created via Create Custom Role). screenshot xperm-AllOn.</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>C26543</t>
+          <t>C26542</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26543</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26542</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -9113,7 +9120,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Only Office User and Time Clock User are non-editable; every other system role (including Administrator) is editable</t>
+          <t>A system role cannot be deleted</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -9123,24 +9130,24 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>Roles-API-Verified (editable flags match live)</t>
+          <t>Roles-API-Verified (all system roles deletable=false)</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>Live roles API: Office User &amp; Time Clock User editable=false; all others (incl. Administrator) editable=true.</t>
+          <t>deletable=false for all system roles (live roles API).</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>C26544</t>
+          <t>C26543</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26544</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26543</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -9153,7 +9160,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Being unable to open Customers does not stop a user from picking a customer when creating a work order</t>
+          <t>Only Office User and Time Clock User are non-editable; every other system role (including Administrator) is editable</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -9163,24 +9170,24 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Roles-API-Verified (editable flags match live)</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>UI: verified via C26385 — a role with Work Orders Create&amp;Edit but NO Customers View cannot open Customers (hidden from nav), yet the New Work Order customer picker still opens and lists existing customers, so a customer can be selected when creating a WO.</t>
+          <t>Live roles API: Office User &amp; Time Clock User editable=false; all others (incl. Administrator) editable=true.</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>C26545</t>
+          <t>C26544</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26545</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26544</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -9193,7 +9200,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>A Page Access toggle that is off overrides the add/edit/delete boxes inside it</t>
+          <t>Being unable to open Customers does not stop a user from picking a customer when creating a work order</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
@@ -9208,19 +9215,19 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>UI: a Page Access toggle that is off overrides inner boxes — a role without reportsPageAccess has no Reports nav entry and /reports is refused (redirects away); a role with Parts Department off hides its 3 child cards (C26407). The Page Access toggle is checked first regardless of inner add/edit/delete.</t>
+          <t>UI: verified via C26385 — a role with Work Orders Create&amp;Edit but NO Customers View cannot open Customers (hidden from nav), yet the New Work Order customer picker still opens and lists existing customers, so a customer can be selected when creating a WO.</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>C26548</t>
+          <t>C26545</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26548</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26545</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -9233,7 +9240,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>View off with Create &amp; Edit on is prevented by the tick-cascade</t>
+          <t>A Page Access toggle that is off overrides the add/edit/delete boxes inside it</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
@@ -9248,19 +9255,19 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>UI/editor: View-off + Create&amp;Edit-on cannot be saved — the tick-cascade (verified C26360/C26362/C26363) auto-ticks View when Create&amp;Edit is ticked, and unticks Create&amp;Edit+Delete when View is unticked, so that invalid combination is impossible in the editor.</t>
+          <t>UI: a Page Access toggle that is off overrides inner boxes — a role without reportsPageAccess has no Reports nav entry and /reports is refused (redirects away); a role with Parts Department off hides its 3 child cards (C26407). The Page Access toggle is checked first regardless of inner add/edit/delete.</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>C26549</t>
+          <t>C26548</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26549</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26548</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -9273,7 +9280,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>AP/AR OFF hides the sensitive customer fields on both the Edit Customer window and the customer overview</t>
+          <t>View off with Create &amp; Edit on is prevented by the tick-cascade</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
@@ -9288,19 +9295,19 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>UI: AP/AR Data OFF hides the sensitive customer fields on the Edit Customer modal (and the financial tabs on the customer overview) — confirmed via Service Advisor (off) vs CustAPAR (on).</t>
+          <t>UI/editor: View-off + Create&amp;Edit-on cannot be saved — the tick-cascade (verified C26360/C26362/C26363) auto-ticks View when Create&amp;Edit is ticked, and unticks Create&amp;Edit+Delete when View is unticked, so that invalid combination is impossible in the editor.</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>C26551</t>
+          <t>C26549</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26551</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26549</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -9313,20 +9320,60 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
+          <t>AP/AR OFF hides the sensitive customer fields on both the Edit Customer window and the customer overview</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>UI: AP/AR Data OFF hides the sensitive customer fields on the Edit Customer modal (and the financial tabs on the customer overview) — confirmed via Service Advisor (off) vs CustAPAR (on).</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>C26551</t>
+        </is>
+      </c>
+      <c r="B205" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26551</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>3553</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Cross-Permission Combinations</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
           <t>Universal clock in/out works even for a user whose role has (almost) no permissions</t>
         </is>
       </c>
-      <c r="F204" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="G204" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="H204" t="inlineStr">
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
         <is>
           <t>UI: the Time Clock User role (only 3 perms: scheduleView/timesheetsView/workOrdersView) still shows the universal Clock In control — universal clock in is not gated by role/permissions.</t>
         </is>
@@ -9537,6 +9584,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B202" r:id="rId201"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B203" r:id="rId202"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B205" r:id="rId204"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9548,7 +9596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10966,25 +11014,25 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>C26526</t>
+          <t>C27731</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26526</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/27731</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3550</v>
+        <v>3549</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Staff Record Settings</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Whether a technician can be scheduled depends on their department, not their role</t>
+          <t>Legacy 'Owner' users become 'Administrator' after migration (Owner merged into Admin)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -10994,24 +11042,24 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Blocked-UI (needs two seeded users + departments)</t>
+          <t>Blocked-UI</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Department-gated scheduling needs live UI.</t>
+          <t>Moved from stub section 3660 into 3549 Migration (was distinct: core 3549 had no legacy-Owner case; Owner is merged into Administrator). Migration LANDING outcome not drivable in this env - needs a real pre-migration 'Owner' user and a migration run (not seedable). Partial confirmation (roles-API): there is NO 'Owner' system role among the 11 shipped system roles, and the Administrator role is editable (roles-matrix-2026-07-13). Full behavior = manual/second-real-user.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>C26527</t>
+          <t>C26526</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26527</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26526</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -11024,7 +11072,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Clocking in on a work order line depends on the per-staff Time Clock setting</t>
+          <t>Whether a technician can be scheduled depends on their department, not their role</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -11034,37 +11082,37 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Blocked-UI (needs two seeded users)</t>
+          <t>Blocked-UI (needs two seeded users + departments)</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Per-staff Time Clock gating needs live UI.</t>
+          <t>Department-gated scheduling needs live UI.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>C26539</t>
+          <t>C26527</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26539</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26527</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3552</v>
+        <v>3550</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>User Feedback Strings</t>
+          <t>Staff Record Settings</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Reassigning a staff member's role updates the row with no success message (billing note in the window)</t>
+          <t>Clocking in on a work order line depends on the per-staff Time Clock setting</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -11074,50 +11122,90 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Blocked-UI (needs live Staff page); billing note not re-captured this pass</t>
+          <t>Blocked-UI (needs two seeded users)</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>No-toast-on-reassign + billing note need live Staff page (EditStaffMember chunk not fetched).</t>
+          <t>Per-staff Time Clock gating needs live UI.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>C26539</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26539</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>3552</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>User Feedback Strings</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Reassigning a staff member's role updates the row with no success message (billing note in the window)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Blocked-UI</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Blocked-UI (needs live Staff page); billing note not re-captured this pass</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>No-toast-on-reassign + billing note need live Staff page (EditStaffMember chunk not fetched).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>C26550</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/26550</t>
         </is>
       </c>
-      <c r="C39" t="n">
+      <c r="C40" t="n">
         <v>3553</v>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Cross-Permission Combinations</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>The last Administrator cannot be left with zero users</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>Blocked-UI</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>Blocked-UI: cannot test the last-Administrator guard on shared staging — the org has 89 users on the Admin role, so the single-last-admin state cannot be created without mass-reassigning real users (destructive/irreversible on a shared env). Product rule; needs an isolated org or DB-level setup. Route to product team to confirm the rule exists.</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>Needs live UI; invariant to confirm.</t>
         </is>
@@ -11163,6 +11251,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId39"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11693,7 +11782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H253"/>
+  <dimension ref="A1:H255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19631,25 +19720,25 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>C26488</t>
+          <t>C27736</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26488</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/27736</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>3546</v>
+        <v>3545</v>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>View History Logs</t>
+          <t>View and Manage AP/AR Data</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>View History Logs ON: work order history and line history are visible (work orders only)</t>
+          <t>The AP/AR cross-cutting toggle is labeled 'View and Manage AP/AR Data'</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -19664,19 +19753,19 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>UI (role with View History Logs ON): the WO detail shows the History (15) tab exposing work order + line history/change events. screenshot hist-HistOn.</t>
+          <t>Moved from stub section 3663 into 3545 (distinct structural check: 3545 had no toggle-label case; parallels the SFD toggle-exists case). Original stub claimed the label 'Manage Accounts Payable and Receivable' - BUILD-WRONG; corrected to the live build label. LABEL VIU-VERIFIED from the shipped build chunk CrossTogglesSection.ChT56hCk.js: 'Cross-Cutting Toggles' card contains 'See Financial Data', 'View and Manage AP/AR Data' (seeApArData), 'View History Logs'.</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>C26489</t>
+          <t>C26488</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26489</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26488</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -19689,7 +19778,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>View History Logs OFF: work order history and line history are hidden (work orders only)</t>
+          <t>View History Logs ON: work order history and line history are visible (work orders only)</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -19704,59 +19793,59 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>UI (role with View History Logs OFF = Time Clock User): the WO detail has NO History tab (Lines/Notes/Timesheets/Stats only) — work order and line history are hidden. screenshot hist-HistOff.</t>
+          <t>UI (role with View History Logs ON): the WO detail shows the History (15) tab exposing work order + line history/change events. screenshot hist-HistOn.</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>C26490</t>
+          <t>C26489</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26490</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26489</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>3547</v>
+        <v>3546</v>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Staff Page Role Assignment</t>
+          <t>View History Logs</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>The Staff role dropdown groups roles into System Roles and Custom Roles</t>
+          <t>View History Logs OFF: work order history and line history are hidden (work orders only)</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Blocked-UI</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>Blocked-UI: the Edit Staff Member Role dropdown (System/Custom grouping) was not reached — the staff row click opened Manage-staff-enrollments. Follow-up: locate the Edit Staff Member action, open the Role selector.</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>11 system roles confirmed in live roles list (was '12'). Grouping labels need live Staff page.</t>
+          <t>UI (role with View History Logs OFF = Time Clock User): the WO detail has NO History tab (Lines/Notes/Timesheets/Stats only) — work order and line history are hidden. screenshot hist-HistOff.</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>C26491</t>
+          <t>C26490</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26491</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26490</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -19769,7 +19858,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>The View Permissions button next to the role selector opens the Permission Summary</t>
+          <t>The Staff role dropdown groups roles into System Roles and Custom Roles</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
@@ -19779,24 +19868,24 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>Blocked-UI: View Permissions eye next to the staff Role selector not reached (same Edit-Staff-Member surface as C26490).</t>
+          <t>Blocked-UI: the Edit Staff Member Role dropdown (System/Custom grouping) was not reached — the staff row click opened Manage-staff-enrollments. Follow-up: locate the Edit Staff Member action, open the Role selector.</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>'View Permissions' confirmed in build. Needs live Staff page.</t>
+          <t>11 system roles confirmed in live roles list (was '12'). Grouping labels need live Staff page.</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>C26492</t>
+          <t>C26491</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26492</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26491</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -19809,34 +19898,34 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Changing a user's role logs them out immediately</t>
+          <t>The View Permissions button next to the role selector opens the Permission Summary</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Blocked-UI</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Blocked-UI: View Permissions eye next to the staff Role selector not reached (same Edit-Staff-Member surface as C26490).</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>API/session: changing a user role logs them out immediately — the prior session is invalidated (409 Session has expired) right after the change.</t>
+          <t>'View Permissions' confirmed in build. Needs live Staff page.</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>C26493</t>
+          <t>C26492</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26493</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26492</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -19849,34 +19938,34 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>If a role change fails, the user keeps their previous role</t>
+          <t>Changing a user's role logs them out immediately</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Blocked-UI</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>Blocked-UI: forcing a failed role change (to confirm the user keeps the prior role) requires inducing a server error on /change; not reproducible on demand this pass.</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>Failed-save path needs live UI.</t>
+          <t>API/session: changing a user role logs them out immediately — the prior session is invalidated (409 Session has expired) right after the change.</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>C26494</t>
+          <t>C26493</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26494</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26493</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -19889,47 +19978,47 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>A logged-in user is logged out immediately when their role changes</t>
+          <t>If a role change fails, the user keeps their previous role</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Blocked-UI</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Blocked-UI: forcing a failed role change (to confirm the user keeps the prior role) requires inducing a server error on /change; not reproducible on demand this pass.</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>API/session: a logged-in user is logged out immediately when their role changes (session invalidated -&gt; 409 on next request).</t>
+          <t>Failed-save path needs live UI.</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>C26495</t>
+          <t>C26494</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26495</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26494</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>3548</v>
+        <v>3547</v>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Per-Role Verification</t>
+          <t>Staff Page Role Assignment</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Administrator: role permissions match the expected set</t>
+          <t>A logged-in user is logged out immediately when their role changes</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
@@ -19939,24 +20028,24 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>Roles-API-Verified (permission set matches the live role); workflow spot-checks Blocked-UI</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>Administrator permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>API/session: a logged-in user is logged out immediately when their role changes (session invalidated -&gt; 409 on next request).</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>C26496</t>
+          <t>C26495</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26496</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26495</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -19969,7 +20058,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Service Manager: role permissions match the expected set</t>
+          <t>Administrator: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
@@ -19984,19 +20073,19 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>Service Manager permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Administrator permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>C26497</t>
+          <t>C26496</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26497</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26496</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -20009,7 +20098,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Senior Service Advisor: role permissions match the expected set</t>
+          <t>Service Manager: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
@@ -20024,19 +20113,19 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>Senior Service Advisor permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Service Manager permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>C26498</t>
+          <t>C26497</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26498</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26497</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -20049,7 +20138,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Service Advisor: role permissions match the expected set</t>
+          <t>Senior Service Advisor: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
@@ -20064,19 +20153,19 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>Service Advisor permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Senior Service Advisor permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>C26499</t>
+          <t>C26498</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26499</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26498</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -20089,7 +20178,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Foreman: role permissions match the expected set</t>
+          <t>Service Advisor: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
@@ -20104,19 +20193,19 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>Foreman permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Service Advisor permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>C26500</t>
+          <t>C26499</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26500</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26499</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -20129,7 +20218,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Technician: role permissions match the expected set</t>
+          <t>Foreman: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
@@ -20144,19 +20233,19 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>Technician permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Foreman permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>C26501</t>
+          <t>C26500</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26501</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26500</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -20169,7 +20258,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Parts Manager: role permissions match the expected set</t>
+          <t>Technician: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
@@ -20184,19 +20273,19 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>Parts Manager permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Technician permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>C26502</t>
+          <t>C26501</t>
         </is>
       </c>
       <c r="B213" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26502</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26501</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -20209,7 +20298,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Parts Technician: role permissions match the expected set</t>
+          <t>Parts Manager: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
@@ -20224,19 +20313,19 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>Parts Technician permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Parts Manager permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>C26503</t>
+          <t>C26502</t>
         </is>
       </c>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26503</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26502</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -20249,7 +20338,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Office User: role permissions match the expected set</t>
+          <t>Parts Technician: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
@@ -20264,19 +20353,19 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>Office User permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Parts Technician permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>C26504</t>
+          <t>C26503</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26504</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26503</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -20289,7 +20378,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Sales Representative: role permissions match the expected set</t>
+          <t>Office User: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
@@ -20304,19 +20393,19 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>Sales Representative permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Office User permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>C26505</t>
+          <t>C26504</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26505</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26504</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -20329,7 +20418,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Time Clock User: role permissions match the expected set</t>
+          <t>Sales Representative: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
@@ -20344,19 +20433,19 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>Time Clock User permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
+          <t>Sales Representative permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>C26506</t>
+          <t>C26505</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26506</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26505</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -20369,7 +20458,7 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Customer portal is on by default only for Service Advisor, Senior Service Advisor, Service Manager and Parts Manager (and Administrator)</t>
+          <t>Time Clock User: role permissions match the expected set</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
@@ -20379,37 +20468,37 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>Roles-API-Verified (matches live per-role customerPortalPageAccess)</t>
+          <t>Roles-API-Verified (permission set matches the live role); workflow spot-checks Blocked-UI</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>customerPortalPageAccess per role confirmed live: on for Admin/SM/SSA/SA/PM; off for the rest (roles-matrix-2026-07-13).</t>
+          <t>Time Clock User permission set confirmed live via GET /api/roles/{id} (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>C26510</t>
+          <t>C26506</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26510</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26506</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>3549</v>
+        <v>3548</v>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Per-Role Verification</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Legacy 'Admin / Administrator' users become 'Administrator' after migration</t>
+          <t>Customer portal is on by default only for Service Advisor, Senior Service Advisor, Service Manager and Parts Manager (and Administrator)</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
@@ -20419,24 +20508,24 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Roles-API-Verified (matches live per-role customerPortalPageAccess)</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>Live roles API: destination system role exists = "Admin" (build name; case prose says Administrator), isEditable=true, 89 users, 42 perms. Migration is a completed historical event; destination state verified (role present, editable with pencil, populated).</t>
+          <t>customerPortalPageAccess per role confirmed live: on for Admin/SM/SSA/SA/PM; off for the rest (roles-matrix-2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>C26511</t>
+          <t>C26510</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26511</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26510</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -20449,7 +20538,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Legacy 'Office' users become 'Office User' after migration</t>
+          <t>Legacy 'Admin / Administrator' users become 'Administrator' after migration</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
@@ -20464,19 +20553,19 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>Live roles API: "Office User" exists, isEditable=false (lock + eye only), 5 users, 23 perms — matches legacy Office -&gt; Office User destination.</t>
+          <t>Live roles API: destination system role exists = "Admin" (build name; case prose says Administrator), isEditable=true, 89 users, 42 perms. Migration is a completed historical event; destination state verified (role present, editable with pencil, populated).</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>C26512</t>
+          <t>C26511</t>
         </is>
       </c>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26512</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26511</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -20489,7 +20578,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>Legacy 'Time Clock' users become 'Time Clock User' after migration</t>
+          <t>Legacy 'Office' users become 'Office User' after migration</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
@@ -20504,19 +20593,19 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>Live roles API: "Time Clock User" exists, isEditable=false (lock + eye only), 11 users, 3 perms — matches legacy Time Clock -&gt; Time Clock User.</t>
+          <t>Live roles API: "Office User" exists, isEditable=false (lock + eye only), 5 users, 23 perms — matches legacy Office -&gt; Office User destination.</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>C26513</t>
+          <t>C26512</t>
         </is>
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26513</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26512</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -20529,7 +20618,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Legacy 'Service Manager' users become 'Service Manager' after migration</t>
+          <t>Legacy 'Time Clock' users become 'Time Clock User' after migration</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
@@ -20544,19 +20633,19 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>Live roles API: "Service Manager" exists, isEditable=true, 3 users, 35 perms.</t>
+          <t>Live roles API: "Time Clock User" exists, isEditable=false (lock + eye only), 11 users, 3 perms — matches legacy Time Clock -&gt; Time Clock User.</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>C26514</t>
+          <t>C26513</t>
         </is>
       </c>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26514</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26513</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -20569,7 +20658,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Legacy 'Senior Service Advisor' users become 'Senior Service Advisor' after migration</t>
+          <t>Legacy 'Service Manager' users become 'Service Manager' after migration</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
@@ -20584,19 +20673,19 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>Live roles API: "Senior Service Advisor" exists, isEditable=true, 8 users, 32 perms.</t>
+          <t>Live roles API: "Service Manager" exists, isEditable=true, 3 users, 35 perms.</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>C26515</t>
+          <t>C26514</t>
         </is>
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26515</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26514</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -20609,7 +20698,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Legacy 'Service Advisor' users become 'Service Advisor' after migration</t>
+          <t>Legacy 'Senior Service Advisor' users become 'Senior Service Advisor' after migration</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
@@ -20624,19 +20713,19 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>Live roles API: "Service Advisor" exists, isEditable=true, 2 users, 26 perms.</t>
+          <t>Live roles API: "Senior Service Advisor" exists, isEditable=true, 8 users, 32 perms.</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>C26516</t>
+          <t>C26515</t>
         </is>
       </c>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26516</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26515</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -20649,7 +20738,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Legacy 'Foreman' users become 'Foreman' after migration</t>
+          <t>Legacy 'Service Advisor' users become 'Service Advisor' after migration</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
@@ -20664,19 +20753,19 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>Live roles API: "Foreman" exists, isEditable=true, 16 users, 23 perms.</t>
+          <t>Live roles API: "Service Advisor" exists, isEditable=true, 2 users, 26 perms.</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>C26517</t>
+          <t>C26516</t>
         </is>
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26517</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26516</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -20689,7 +20778,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Legacy 'Technician' users become 'Technician' after migration</t>
+          <t>Legacy 'Foreman' users become 'Foreman' after migration</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
@@ -20704,19 +20793,19 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>Live roles API: "Technician" exists, isEditable=true, 66 users, 6 perms, view_mode tech (confirmed via role detail) — matches legacy Technician destination.</t>
+          <t>Live roles API: "Foreman" exists, isEditable=true, 16 users, 23 perms.</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>C26518</t>
+          <t>C26517</t>
         </is>
       </c>
       <c r="B226" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26518</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26517</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -20729,7 +20818,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Legacy 'Parts Manager' users become 'Parts Manager' after migration</t>
+          <t>Legacy 'Technician' users become 'Technician' after migration</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
@@ -20744,19 +20833,19 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>Live roles API: "Parts Manager" exists, isEditable=true, 4 users, 31 perms.</t>
+          <t>Live roles API: "Technician" exists, isEditable=true, 66 users, 6 perms, view_mode tech (confirmed via role detail) — matches legacy Technician destination.</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>C26519</t>
+          <t>C26518</t>
         </is>
       </c>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26519</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26518</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -20769,7 +20858,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Legacy 'Parts Tech / Parts Technician' users become 'Parts Technician' after migration</t>
+          <t>Legacy 'Parts Manager' users become 'Parts Manager' after migration</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
@@ -20784,19 +20873,19 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>Live roles API: "Parts Technician" exists, isEditable=true, 10 users, 19 perms — matches legacy Parts Tech -&gt; Parts Technician.</t>
+          <t>Live roles API: "Parts Manager" exists, isEditable=true, 4 users, 31 perms.</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>C26520</t>
+          <t>C26519</t>
         </is>
       </c>
       <c r="B228" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26520</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26519</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -20809,7 +20898,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Legacy 'Sales Representative' users become 'Sales Representative' after migration</t>
+          <t>Legacy 'Parts Tech / Parts Technician' users become 'Parts Technician' after migration</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
@@ -20824,19 +20913,19 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>Live roles API: "Sales Representative" exists, isEditable=true, 15 users, 4 perms.</t>
+          <t>Live roles API: "Parts Technician" exists, isEditable=true, 10 users, 19 perms — matches legacy Parts Tech -&gt; Parts Technician.</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>C26525</t>
+          <t>C26520</t>
         </is>
       </c>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26525</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26520</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -20849,7 +20938,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Changing a user's role logs that user out and forces them to log in again</t>
+          <t>Legacy 'Sales Representative' users become 'Sales Representative' after migration</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
@@ -20864,72 +20953,72 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>UI/API: after an admin changed the Tech user role, the user existing session returned 409 "Session has expired." on the next call — the role change logs the user out and forces re-login.</t>
+          <t>Live roles API: "Sales Representative" exists, isEditable=true, 15 users, 4 perms.</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>C26526</t>
+          <t>C26525</t>
         </is>
       </c>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26526</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26525</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>3550</v>
+        <v>3549</v>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Staff Record Settings</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Whether a technician can be scheduled depends on their department, not their role</t>
+          <t>Changing a user's role logs that user out and forces them to log in again</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>Blocked-UI</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>Blocked-UI (needs two seeded users + departments)</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>Department-gated scheduling needs live UI.</t>
+          <t>UI/API: after an admin changed the Tech user role, the user existing session returned 409 "Session has expired." on the next call — the role change logs the user out and forces re-login.</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>C26527</t>
+          <t>C27731</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26527</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/27731</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>3550</v>
+        <v>3549</v>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Staff Record Settings</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Clocking in on a work order line depends on the per-staff Time Clock setting</t>
+          <t>Legacy 'Owner' users become 'Administrator' after migration (Owner merged into Admin)</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
@@ -20939,24 +21028,24 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>Blocked-UI (needs two seeded users)</t>
+          <t>Blocked-UI</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>Per-staff Time Clock gating needs live UI.</t>
+          <t>Moved from stub section 3660 into 3549 Migration (was distinct: core 3549 had no legacy-Owner case; Owner is merged into Administrator). Migration LANDING outcome not drivable in this env - needs a real pre-migration 'Owner' user and a migration run (not seedable). Partial confirmation (roles-API): there is NO 'Owner' system role among the 11 shipped system roles, and the Administrator role is editable (roles-matrix-2026-07-13). Full behavior = manual/second-real-user.</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>C26528</t>
+          <t>C26526</t>
         </is>
       </c>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26528</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26526</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -20969,114 +21058,114 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>The universal clock in / out is available to any active staff member, whatever their role</t>
+          <t>Whether a technician can be scheduled depends on their department, not their role</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Blocked-UI</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Blocked-UI (needs two seeded users + departments)</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>UI: the universal Clock In control appears in the top bar for every role observed (Admin, Technician, Time Clock User) — available to any active staff member whatever their role.</t>
+          <t>Department-gated scheduling needs live UI.</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>C26529</t>
+          <t>C26527</t>
         </is>
       </c>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26529</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26527</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>3551</v>
+        <v>3550</v>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>QuickBooks Relocation</t>
+          <t>Staff Record Settings</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>QuickBooks settings appear under Integrations when the Integrations sub-toggle is ON</t>
+          <t>Clocking in on a work order line depends on the per-staff Time Clock setting</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Deviation/Finding</t>
+          <t>Blocked-UI</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>Deviation-vs-old-case: build has QuickBooks under Integrations, not Finance</t>
+          <t>Blocked-UI (needs two seeded users)</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>Route metadata: Integrations gates IBS/Open API/QuickBooks; Finance gates Payment Methods/Taxes (no QuickBooks). QuickBooks is under Integrations in the build.</t>
+          <t>Per-staff Time Clock gating needs live UI.</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>C26530</t>
+          <t>C26528</t>
         </is>
       </c>
       <c r="B234" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26530</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26528</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>3551</v>
+        <v>3550</v>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>QuickBooks Relocation</t>
+          <t>Staff Record Settings</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>QuickBooks settings are hidden when the Integrations sub-toggle is OFF</t>
+          <t>The universal clock in / out is available to any active staff member, whatever their role</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>Deviation/Finding</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>Deviation-vs-old-case: QuickBooks gated by Integrations, not Finance</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>QuickBooks gated by settingsIntegrations in the build.</t>
+          <t>UI: the universal Clock In control appears in the top bar for every role observed (Admin, Technician, Time Clock User) — available to any active staff member whatever their role.</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>C26531</t>
+          <t>C26529</t>
         </is>
       </c>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26531</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26529</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -21089,7 +21178,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>The Integrations settings section is present and hosts QuickBooks, IBS and Open API</t>
+          <t>QuickBooks settings appear under Integrations when the Integrations sub-toggle is ON</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
@@ -21099,104 +21188,104 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>Deviation-vs-old-case: Integrations IS present in build (old case said removed)</t>
+          <t>Deviation-vs-old-case: build has QuickBooks under Integrations, not Finance</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>settingsIntegrations gates IBS/Open API/QuickBooks; the Settings 'Integrations' sub-toggle exists. Integrations is present in the build.</t>
+          <t>Route metadata: Integrations gates IBS/Open API/QuickBooks; Finance gates Payment Methods/Taxes (no QuickBooks). QuickBooks is under Integrations in the build.</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>C26532</t>
+          <t>C26530</t>
         </is>
       </c>
       <c r="B236" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26532</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26530</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>3552</v>
+        <v>3551</v>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>User Feedback Strings</t>
+          <t>QuickBooks Relocation</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Create success message wording</t>
+          <t>QuickBooks settings are hidden when the Integrations sub-toggle is OFF</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Deviation/Finding</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>Verified-Label (build)</t>
+          <t>Deviation-vs-old-case: QuickBooks gated by Integrations, not Finance</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>'Role created successfully.' confirmed in build.</t>
+          <t>QuickBooks gated by settingsIntegrations in the build.</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>C26533</t>
+          <t>C26531</t>
         </is>
       </c>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26533</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26531</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>3552</v>
+        <v>3551</v>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>User Feedback Strings</t>
+          <t>QuickBooks Relocation</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Update success message wording</t>
+          <t>The Integrations settings section is present and hosts QuickBooks, IBS and Open API</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Deviation/Finding</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>Verified-Label (build)</t>
+          <t>Deviation-vs-old-case: Integrations IS present in build (old case said removed)</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>'Role updated successfully.' confirmed in build.</t>
+          <t>settingsIntegrations gates IBS/Open API/QuickBooks; the Settings 'Integrations' sub-toggle exists. Integrations is present in the build.</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>C26534</t>
+          <t>C26532</t>
         </is>
       </c>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26534</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26532</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -21209,7 +21298,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Deleting a custom role with 0 users shows a confirmation dialog</t>
+          <t>Create success message wording</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
@@ -21219,24 +21308,24 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Verified-Label (build)</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>UI: deleting a 0-user custom role opens dialog "Confirmation — Are you sure you want to delete this role? This action cannot be undone." [Cancel|Delete]. screenshot delete-confirm-dialog.</t>
+          <t>'Role created successfully.' confirmed in build.</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>C26535</t>
+          <t>C26533</t>
         </is>
       </c>
       <c r="B239" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26535</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26533</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -21249,7 +21338,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Deleting a custom role that has users is blocked</t>
+          <t>Update success message wording</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
@@ -21259,24 +21348,24 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Verified-Label (build)</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>UI: a custom role with users (Parth Cust1, 1 user) has no Delete option in its 3-dot menu — deletion is blocked.</t>
+          <t>'Role updated successfully.' confirmed in build.</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>C26536</t>
+          <t>C26534</t>
         </is>
       </c>
       <c r="B240" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26536</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26534</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -21289,7 +21378,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Turning See Financial Data on shows a confirmation dialog</t>
+          <t>Deleting a custom role with 0 users shows a confirmation dialog</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -21299,24 +21388,24 @@
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>Verified-Label (build)</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>'Enable See Financial Data?' + Cancel/Enable confirmed in build (FinancialDataConfirmModal).</t>
+          <t>UI: deleting a 0-user custom role opens dialog "Confirmation — Are you sure you want to delete this role? This action cannot be undone." [Cancel|Delete]. screenshot delete-confirm-dialog.</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>C26537</t>
+          <t>C26535</t>
         </is>
       </c>
       <c r="B241" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26537</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26535</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -21329,7 +21418,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Creating a role with no name is blocked with a required-field error</t>
+          <t>Deleting a custom role that has users is blocked</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
@@ -21344,19 +21433,19 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>UI: creating a role with no name is blocked — Create disabled and inline "Role name is a required field" error when the field is touched/cleared.</t>
+          <t>UI: a custom role with users (Parth Cust1, 1 user) has no Delete option in its 3-dot menu — deletion is blocked.</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>C26538</t>
+          <t>C26536</t>
         </is>
       </c>
       <c r="B242" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26538</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26536</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -21369,7 +21458,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Creating a role with the same permissions as an existing role shows a 'similar role' warning</t>
+          <t>Turning See Financial Data on shows a confirmation dialog</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -21379,24 +21468,24 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Verified-Label (build)</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>UI: creating a role with the same permissions as an existing role shows "Similar role already exists" warning with "Create Anyway" (SimilarRoleWarningModal, keyed on identical permissions).</t>
+          <t>'Enable See Financial Data?' + Cancel/Enable confirmed in build (FinancialDataConfirmModal).</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>C26539</t>
+          <t>C26537</t>
         </is>
       </c>
       <c r="B243" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26539</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26537</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -21409,47 +21498,47 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Reassigning a staff member's role updates the row with no success message (billing note in the window)</t>
+          <t>Creating a role with no name is blocked with a required-field error</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>Blocked-UI</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>Blocked-UI (needs live Staff page); billing note not re-captured this pass</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>No-toast-on-reassign + billing note need live Staff page (EditStaffMember chunk not fetched).</t>
+          <t>UI: creating a role with no name is blocked — Create disabled and inline "Role name is a required field" error when the field is touched/cleared.</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>C26540</t>
+          <t>C26538</t>
         </is>
       </c>
       <c r="B244" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26540</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26538</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>3553</v>
+        <v>3552</v>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Cross-Permission Combinations</t>
+          <t>User Feedback Strings</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>A role with all permissions off blocks the user from every feature</t>
+          <t>Creating a role with the same permissions as an existing role shows a 'similar role' warning</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
@@ -21464,59 +21553,59 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>UI: a near-minimal custom role (only scheduleView) shows a minimal nav (just Schedule + Clock In); navigating to /reports or /administration/staff is refused and redirects to /schedule. (A truly all-off role cannot be saved — Create is disabled at zero perms, C26335 — so the practical minimum is one feature perm; that user is blocked from every other feature.) screenshot xperm-MinRole.</t>
+          <t>UI: creating a role with the same permissions as an existing role shows "Similar role already exists" warning with "Create Anyway" (SimilarRoleWarningModal, keyed on identical permissions).</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>C26541</t>
+          <t>C26539</t>
         </is>
       </c>
       <c r="B245" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26541</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26539</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>3553</v>
+        <v>3552</v>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Cross-Permission Combinations</t>
+          <t>User Feedback Strings</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>A role with all permissions on behaves like Administrator but is still a custom role</t>
+          <t>Reassigning a staff member's role updates the row with no success message (billing note in the window)</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Blocked-UI</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Blocked-UI (needs live Staff page); billing note not re-captured this pass</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>UI: an all-permissions custom role (42 perms, all cross-toggles on, type Custom) behaves like Administrator — full nav (Work Orders/Schedule/Customers/Parts/Reports), /reports and /administration/staff accessible — yet it is a Custom role (created via Create Custom Role). screenshot xperm-AllOn.</t>
+          <t>No-toast-on-reassign + billing note need live Staff page (EditStaffMember chunk not fetched).</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>C26542</t>
+          <t>C26540</t>
         </is>
       </c>
       <c r="B246" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26542</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26540</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -21529,7 +21618,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>A system role cannot be deleted</t>
+          <t>A role with all permissions off blocks the user from every feature</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
@@ -21539,24 +21628,24 @@
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>Roles-API-Verified (all system roles deletable=false)</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>deletable=false for all system roles (live roles API).</t>
+          <t>UI: a near-minimal custom role (only scheduleView) shows a minimal nav (just Schedule + Clock In); navigating to /reports or /administration/staff is refused and redirects to /schedule. (A truly all-off role cannot be saved — Create is disabled at zero perms, C26335 — so the practical minimum is one feature perm; that user is blocked from every other feature.) screenshot xperm-MinRole.</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>C26543</t>
+          <t>C26541</t>
         </is>
       </c>
       <c r="B247" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26543</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26541</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -21569,7 +21658,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Only Office User and Time Clock User are non-editable; every other system role (including Administrator) is editable</t>
+          <t>A role with all permissions on behaves like Administrator but is still a custom role</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
@@ -21579,24 +21668,24 @@
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>Roles-API-Verified (editable flags match live)</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>Live roles API: Office User &amp; Time Clock User editable=false; all others (incl. Administrator) editable=true.</t>
+          <t>UI: an all-permissions custom role (42 perms, all cross-toggles on, type Custom) behaves like Administrator — full nav (Work Orders/Schedule/Customers/Parts/Reports), /reports and /administration/staff accessible — yet it is a Custom role (created via Create Custom Role). screenshot xperm-AllOn.</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>C26544</t>
+          <t>C26542</t>
         </is>
       </c>
       <c r="B248" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26544</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26542</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -21609,7 +21698,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Being unable to open Customers does not stop a user from picking a customer when creating a work order</t>
+          <t>A system role cannot be deleted</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -21619,24 +21708,24 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Roles-API-Verified (all system roles deletable=false)</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>UI: verified via C26385 — a role with Work Orders Create&amp;Edit but NO Customers View cannot open Customers (hidden from nav), yet the New Work Order customer picker still opens and lists existing customers, so a customer can be selected when creating a WO.</t>
+          <t>deletable=false for all system roles (live roles API).</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>C26545</t>
+          <t>C26543</t>
         </is>
       </c>
       <c r="B249" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26545</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26543</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -21649,7 +21738,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>A Page Access toggle that is off overrides the add/edit/delete boxes inside it</t>
+          <t>Only Office User and Time Clock User are non-editable; every other system role (including Administrator) is editable</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -21659,24 +21748,24 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Roles-API-Verified (editable flags match live)</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>UI: a Page Access toggle that is off overrides inner boxes — a role without reportsPageAccess has no Reports nav entry and /reports is refused (redirects away); a role with Parts Department off hides its 3 child cards (C26407). The Page Access toggle is checked first regardless of inner add/edit/delete.</t>
+          <t>Live roles API: Office User &amp; Time Clock User editable=false; all others (incl. Administrator) editable=true.</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>C26548</t>
+          <t>C26544</t>
         </is>
       </c>
       <c r="B250" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26548</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26544</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -21689,7 +21778,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>View off with Create &amp; Edit on is prevented by the tick-cascade</t>
+          <t>Being unable to open Customers does not stop a user from picking a customer when creating a work order</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -21704,19 +21793,19 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>UI/editor: View-off + Create&amp;Edit-on cannot be saved — the tick-cascade (verified C26360/C26362/C26363) auto-ticks View when Create&amp;Edit is ticked, and unticks Create&amp;Edit+Delete when View is unticked, so that invalid combination is impossible in the editor.</t>
+          <t>UI: verified via C26385 — a role with Work Orders Create&amp;Edit but NO Customers View cannot open Customers (hidden from nav), yet the New Work Order customer picker still opens and lists existing customers, so a customer can be selected when creating a WO.</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>C26549</t>
+          <t>C26545</t>
         </is>
       </c>
       <c r="B251" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26549</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26545</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -21729,7 +21818,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>AP/AR OFF hides the sensitive customer fields on both the Edit Customer window and the customer overview</t>
+          <t>A Page Access toggle that is off overrides the add/edit/delete boxes inside it</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -21744,19 +21833,19 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>UI: AP/AR Data OFF hides the sensitive customer fields on the Edit Customer modal (and the financial tabs on the customer overview) — confirmed via Service Advisor (off) vs CustAPAR (on).</t>
+          <t>UI: a Page Access toggle that is off overrides inner boxes — a role without reportsPageAccess has no Reports nav entry and /reports is refused (redirects away); a role with Parts Department off hides its 3 child cards (C26407). The Page Access toggle is checked first regardless of inner add/edit/delete.</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>C26550</t>
+          <t>C26548</t>
         </is>
       </c>
       <c r="B252" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26550</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26548</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -21769,34 +21858,34 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>The last Administrator cannot be left with zero users</t>
+          <t>View off with Create &amp; Edit on is prevented by the tick-cascade</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Blocked-UI</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>Blocked-UI: cannot test the last-Administrator guard on shared staging — the org has 89 users on the Admin role, so the single-last-admin state cannot be created without mass-reassigning real users (destructive/irreversible on a shared env). Product rule; needs an isolated org or DB-level setup. Route to product team to confirm the rule exists.</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>Needs live UI; invariant to confirm.</t>
+          <t>UI/editor: View-off + Create&amp;Edit-on cannot be saved — the tick-cascade (verified C26360/C26362/C26363) auto-ticks View when Create&amp;Edit is ticked, and unticks Create&amp;Edit+Delete when View is unticked, so that invalid combination is impossible in the editor.</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>C26551</t>
+          <t>C26549</t>
         </is>
       </c>
       <c r="B253" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/26551</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26549</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -21809,20 +21898,100 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
+          <t>AP/AR OFF hides the sensitive customer fields on both the Edit Customer window and the customer overview</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>UI: AP/AR Data OFF hides the sensitive customer fields on the Edit Customer modal (and the financial tabs on the customer overview) — confirmed via Service Advisor (off) vs CustAPAR (on).</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>C26550</t>
+        </is>
+      </c>
+      <c r="B254" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26550</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>3553</v>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Cross-Permission Combinations</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>The last Administrator cannot be left with zero users</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Blocked-UI</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Blocked-UI: cannot test the last-Administrator guard on shared staging — the org has 89 users on the Admin role, so the single-last-admin state cannot be created without mass-reassigning real users (destructive/irreversible on a shared env). Product rule; needs an isolated org or DB-level setup. Route to product team to confirm the rule exists.</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>Needs live UI; invariant to confirm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>C26551</t>
+        </is>
+      </c>
+      <c r="B255" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/26551</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>3553</v>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Cross-Permission Combinations</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
           <t>Universal clock in/out works even for a user whose role has (almost) no permissions</t>
         </is>
       </c>
-      <c r="F253" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="G253" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="H253" t="inlineStr">
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
         <is>
           <t>UI: the Time Clock User role (only 3 perms: scheduleView/timesheetsView/workOrdersView) still shows the universal Clock In control — universal clock in is not gated by role/permissions.</t>
         </is>
@@ -22082,6 +22251,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B251" r:id="rId250"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B252" r:id="rId251"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B255" r:id="rId254"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Custom Roles: delete 5 not-valid section-3658 stubs; finalize canonical wording+VIU state
- Deleted C27729/C27730/C27732/C27734/C27738 via TestRail delete_case (QA-lead
  authorized); each verified gone. Section 3658 subtree now empty.
- Finalized WORDING-VIU-STATE-2026-07-13.md as canonical cold-resume doc
  (final tally 254 = 204 Verified / 39 Blocked-UI / 11 Deviation).
- Synced CLAUDE.md Custom Roles entry; updated audit log, resolution doc,
  Blockers Tracker, and regenerated WordingVIU workbook to 254.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/custom-roles-run/CustomRoles_WordingVIU_2026-07-13.xlsx
+++ b/build/custom-roles-run/CustomRoles_WordingVIU_2026-07-13.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -462,7 +462,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TestRail push: all 252 core cases (sections 3528–3553) updated via update_case, 200/200, 0 errors (wording pass).</t>
+          <t>TestRail push: all 252 core cases (sections 3528–3553) updated via update_case, 200/200, 0 errors (wording pass); + 2 valid stubs moved into 3527 and reworded/pushed = 254 cases total in this workbook.</t>
         </is>
       </c>
     </row>
@@ -476,163 +476,178 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Section 3658 dedupe: 3 duplicates deleted (C27735, C27733, C27737).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Section 3658 resolution 2026-07-13: 2 valid stubs MOVED into 3527 sub-sections + reworded/pushed (C27731-&gt;3549 Migration, C27736-&gt;3545 View and Manage AP/AR Data); 5 left in 3658 for QA-lead decision (C27729, C27730, C27732, C27734, C27738 - redundant or build-wrong). See section-3658-resolution-2026-07-13.md.</t>
+          <t>Section 3658 stub tree FULLY RESOLVED 2026-07-13: original 10 stubs = 3 duplicates deleted early (C27735, C27733, C27737) + 2 valid stubs MOVED into 3527 sub-sections + reworded/pushed (C27731-&gt;3549 Migration, C27736-&gt;3545 View and Manage AP/AR Data) + 5 not-valid stubs DELETED (C27729, C27730, C27732, C27734, C27738 - redundant or build-wrong, QA-lead authorized). Section 3658 subtree (3658–3665) now EMPTY. See section-3658-resolution-2026-07-13.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Bucket</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Count</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Bucket</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>204</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>VIU-Verified</t>
+          <t>Blocked-UI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>204</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Blocked-UI</t>
+          <t>Deviation/Finding</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Blocked-UI</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
           <t>Deviation/Finding</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Roles List Page (3528)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>18</v>
+      </c>
+      <c r="C15" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Area</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Blocked-UI</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Deviation/Finding</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Roles List Page (3528)</t>
+          <t>Create Custom Role (3529)</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Create Custom Role (3529)</t>
+          <t>Edit Role (3530)</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Edit Role (3530)</t>
+          <t>Delete Role (3531)</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
@@ -644,20 +659,20 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Delete Role (3531)</t>
+          <t>Permission Summary (3532)</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -672,14 +687,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Permission Summary (3532)</t>
+          <t>CRUD Cascade Rules (3533)</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -688,61 +703,61 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CRUD Cascade Rules (3533)</t>
+          <t>Work Orders Permissions (3534)</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Work Orders Permissions (3534)</t>
+          <t>Work Order Lines Permissions (3535)</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Work Order Lines Permissions (3535)</t>
+          <t>Schedule Permissions (3536)</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C23" t="n">
         <v>3</v>
@@ -754,20 +769,20 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Schedule Permissions (3536)</t>
+          <t>Customer Management Permissions (3537)</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -776,20 +791,20 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Customer Management Permissions (3537)</t>
+          <t>Parts Department Permissions (3538)</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -798,64 +813,64 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Parts Department Permissions (3538)</t>
+          <t>Invoicing and Payments Permissions (3539)</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Invoicing and Payments Permissions (3539)</t>
+          <t>Timesheets Permissions (3540)</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>6</v>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Timesheets Permissions (3540)</t>
+          <t>Page Access Toggles (3541)</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -864,20 +879,20 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Page Access Toggles (3541)</t>
+          <t>Settings Access (3542)</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -886,64 +901,64 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Settings Access (3542)</t>
+          <t>View Mode (3543)</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>View Mode (3543)</t>
+          <t>See Financial Data (3544)</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>See Financial Data (3544)</t>
+          <t>View and Manage AP/AR Data (3545)</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
@@ -952,20 +967,20 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>View and Manage AP/AR Data (3545)</t>
+          <t>View History Logs (3546)</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -974,20 +989,20 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>View History Logs (3546)</t>
+          <t>Staff Page Role Assignment (3547)</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -996,20 +1011,20 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Staff Page Role Assignment (3547)</t>
+          <t>Per-Role Verification (3548)</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -1018,20 +1033,20 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Per-Role Verification (3548)</t>
+          <t>Migration (3549)</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>12</v>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
@@ -1040,20 +1055,20 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Migration (3549)</t>
+          <t>Staff Record Settings (3550)</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -1062,23 +1077,23 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Staff Record Settings (3550)</t>
+          <t>QuickBooks Relocation (3551)</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
@@ -1090,33 +1105,33 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>QuickBooks Relocation (3551)</t>
+          <t>User Feedback Strings (3552)</t>
         </is>
       </c>
       <c r="B39" t="n">
+        <v>7</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
         <v>0</v>
-      </c>
-      <c r="C39" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" t="n">
-        <v>3</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>User Feedback Strings (3552)</t>
+          <t>Cross-Permission Combinations (3553)</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C40" t="n">
         <v>1</v>
@@ -1128,28 +1143,6 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Cross-Permission Combinations (3553)</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>9</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
-        <v>0</v>
-      </c>
-      <c r="E41" t="n">
-        <v>0</v>
-      </c>
-      <c r="F41" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>